<commit_message>
up to date on config details
</commit_message>
<xml_diff>
--- a/src/config/midas_config_values.xlsx
+++ b/src/config/midas_config_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/james/Documents/code/midas-alt/src/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE78FA91-C5F8-3845-B782-703E8ECDC042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A26520C-FD58-5E49-8F5F-2067945475D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="500" windowWidth="39880" windowHeight="28300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80" yWindow="500" windowWidth="39880" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>